<commit_message>
Finish forum, Add CSS page message and edit journal du groupe
</commit_message>
<xml_diff>
--- a/planning/Journal_planification_du_groupe.xlsx
+++ b/planning/Journal_planification_du_groupe.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilstan.sanquer\Desktop\Github\SquidTchat\planning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6CB8D2D3-FFC1-493C-B9A0-524A84A15055}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A13A662-9BFF-41C4-9B4D-77762DF6EDB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{80F6D908-82BF-40D3-B5DB-CACD124443E4}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
   <si>
     <t>Jour</t>
   </si>
@@ -386,6 +386,154 @@
         <scheme val="minor"/>
       </rPr>
       <t>Wilstan</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">• 1h : Développement du CSS - Messagerie privée : </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Wilstan</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+• 1h : Mise à jour du cahier de recette :</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Raphaël</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+• 30 min : Optimisation du filtre des pseudos : </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Raphaël</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+• 2h : Implémentation de la recherche utilisateur – Messagerie privée :</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Jean</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+• 3h : Intégration JavaScript – Messagerie privée : </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Wilstan</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+• 30 min : Réunion de planification – Étapes suivantes :</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Wilstan, Jean, Raphaël</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+• 2h : Gestion de la déconnexion et libération des pseudos : </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Jean</t>
     </r>
   </si>
 </sst>
@@ -557,32 +705,56 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -608,30 +780,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
@@ -658,27 +806,20 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1018,187 +1159,187 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
-      <c r="P1" s="18"/>
-      <c r="Q1" s="18"/>
-      <c r="R1" s="18"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+      <c r="M1" s="7"/>
+      <c r="N1" s="7"/>
+      <c r="O1" s="7"/>
+      <c r="P1" s="7"/>
+      <c r="Q1" s="7"/>
+      <c r="R1" s="7"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A2" s="18"/>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
-      <c r="J2" s="18"/>
-      <c r="K2" s="18"/>
-      <c r="L2" s="18"/>
-      <c r="M2" s="18"/>
-      <c r="N2" s="18"/>
-      <c r="O2" s="18"/>
-      <c r="P2" s="18"/>
-      <c r="Q2" s="18"/>
-      <c r="R2" s="18"/>
+      <c r="A2" s="7"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
+      <c r="K2" s="7"/>
+      <c r="L2" s="7"/>
+      <c r="M2" s="7"/>
+      <c r="N2" s="7"/>
+      <c r="O2" s="7"/>
+      <c r="P2" s="7"/>
+      <c r="Q2" s="7"/>
+      <c r="R2" s="7"/>
     </row>
     <row r="3" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19" t="s">
+      <c r="B3" s="8"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="9" t="s">
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="11"/>
-      <c r="I3" s="9" t="s">
+      <c r="H3" s="19"/>
+      <c r="I3" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="J3" s="10"/>
-      <c r="K3" s="10"/>
-      <c r="L3" s="10"/>
-      <c r="M3" s="10"/>
-      <c r="N3" s="10"/>
-      <c r="O3" s="10"/>
-      <c r="P3" s="10"/>
-      <c r="Q3" s="10"/>
-      <c r="R3" s="11"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="18"/>
+      <c r="M3" s="18"/>
+      <c r="N3" s="18"/>
+      <c r="O3" s="18"/>
+      <c r="P3" s="18"/>
+      <c r="Q3" s="18"/>
+      <c r="R3" s="19"/>
     </row>
     <row r="4" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="19"/>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="12"/>
-      <c r="H4" s="14"/>
-      <c r="I4" s="12"/>
-      <c r="J4" s="13"/>
-      <c r="K4" s="13"/>
-      <c r="L4" s="13"/>
-      <c r="M4" s="13"/>
-      <c r="N4" s="13"/>
-      <c r="O4" s="13"/>
-      <c r="P4" s="13"/>
-      <c r="Q4" s="13"/>
-      <c r="R4" s="14"/>
+      <c r="A4" s="8"/>
+      <c r="B4" s="8"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="20"/>
+      <c r="H4" s="22"/>
+      <c r="I4" s="20"/>
+      <c r="J4" s="21"/>
+      <c r="K4" s="21"/>
+      <c r="L4" s="21"/>
+      <c r="M4" s="21"/>
+      <c r="N4" s="21"/>
+      <c r="O4" s="21"/>
+      <c r="P4" s="21"/>
+      <c r="Q4" s="21"/>
+      <c r="R4" s="22"/>
     </row>
     <row r="5" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="19"/>
-      <c r="B5" s="19"/>
-      <c r="C5" s="19"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="19"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="14"/>
-      <c r="I5" s="12"/>
-      <c r="J5" s="13"/>
-      <c r="K5" s="13"/>
-      <c r="L5" s="13"/>
-      <c r="M5" s="13"/>
-      <c r="N5" s="13"/>
-      <c r="O5" s="13"/>
-      <c r="P5" s="13"/>
-      <c r="Q5" s="13"/>
-      <c r="R5" s="14"/>
+      <c r="A5" s="8"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="20"/>
+      <c r="H5" s="22"/>
+      <c r="I5" s="20"/>
+      <c r="J5" s="21"/>
+      <c r="K5" s="21"/>
+      <c r="L5" s="21"/>
+      <c r="M5" s="21"/>
+      <c r="N5" s="21"/>
+      <c r="O5" s="21"/>
+      <c r="P5" s="21"/>
+      <c r="Q5" s="21"/>
+      <c r="R5" s="22"/>
     </row>
     <row r="6" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="19"/>
-      <c r="B6" s="19"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="12"/>
-      <c r="H6" s="14"/>
-      <c r="I6" s="12"/>
-      <c r="J6" s="13"/>
-      <c r="K6" s="13"/>
-      <c r="L6" s="13"/>
-      <c r="M6" s="13"/>
-      <c r="N6" s="13"/>
-      <c r="O6" s="13"/>
-      <c r="P6" s="13"/>
-      <c r="Q6" s="13"/>
-      <c r="R6" s="14"/>
+      <c r="A6" s="8"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="20"/>
+      <c r="H6" s="22"/>
+      <c r="I6" s="20"/>
+      <c r="J6" s="21"/>
+      <c r="K6" s="21"/>
+      <c r="L6" s="21"/>
+      <c r="M6" s="21"/>
+      <c r="N6" s="21"/>
+      <c r="O6" s="21"/>
+      <c r="P6" s="21"/>
+      <c r="Q6" s="21"/>
+      <c r="R6" s="22"/>
     </row>
     <row r="7" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="19"/>
-      <c r="B7" s="19"/>
-      <c r="C7" s="19"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="19"/>
-      <c r="F7" s="19"/>
-      <c r="G7" s="12"/>
-      <c r="H7" s="14"/>
-      <c r="I7" s="12"/>
-      <c r="J7" s="13"/>
-      <c r="K7" s="13"/>
-      <c r="L7" s="13"/>
-      <c r="M7" s="13"/>
-      <c r="N7" s="13"/>
-      <c r="O7" s="13"/>
-      <c r="P7" s="13"/>
-      <c r="Q7" s="13"/>
-      <c r="R7" s="14"/>
+      <c r="A7" s="8"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="20"/>
+      <c r="H7" s="22"/>
+      <c r="I7" s="20"/>
+      <c r="J7" s="21"/>
+      <c r="K7" s="21"/>
+      <c r="L7" s="21"/>
+      <c r="M7" s="21"/>
+      <c r="N7" s="21"/>
+      <c r="O7" s="21"/>
+      <c r="P7" s="21"/>
+      <c r="Q7" s="21"/>
+      <c r="R7" s="22"/>
     </row>
     <row r="8" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="19"/>
-      <c r="B8" s="19"/>
-      <c r="C8" s="19"/>
-      <c r="D8" s="19"/>
-      <c r="E8" s="19"/>
-      <c r="F8" s="19"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="15"/>
-      <c r="J8" s="16"/>
-      <c r="K8" s="16"/>
-      <c r="L8" s="16"/>
-      <c r="M8" s="16"/>
-      <c r="N8" s="16"/>
-      <c r="O8" s="16"/>
-      <c r="P8" s="16"/>
-      <c r="Q8" s="16"/>
-      <c r="R8" s="17"/>
+      <c r="A8" s="8"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="25"/>
+      <c r="I8" s="23"/>
+      <c r="J8" s="24"/>
+      <c r="K8" s="24"/>
+      <c r="L8" s="24"/>
+      <c r="M8" s="24"/>
+      <c r="N8" s="24"/>
+      <c r="O8" s="24"/>
+      <c r="P8" s="24"/>
+      <c r="Q8" s="24"/>
+      <c r="R8" s="25"/>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A9" s="8">
+      <c r="A9" s="10">
         <v>46094</v>
       </c>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1" t="s">
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="2" t="s">
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="3" t="s">
         <v>5</v>
       </c>
       <c r="H9" s="4"/>
@@ -1216,14 +1357,14 @@
       <c r="R9" s="28"/>
     </row>
     <row r="10" spans="1:18" ht="84" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
+      <c r="A10" s="9"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
       <c r="G10" s="5"/>
-      <c r="H10" s="7"/>
+      <c r="H10" s="6"/>
       <c r="I10" s="29"/>
       <c r="J10" s="30"/>
       <c r="K10" s="30"/>
@@ -1236,17 +1377,17 @@
       <c r="R10" s="31"/>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A11" s="20">
+      <c r="A11" s="11">
         <v>46098</v>
       </c>
-      <c r="B11" s="21"/>
-      <c r="C11" s="22"/>
-      <c r="D11" s="1" t="s">
+      <c r="B11" s="12"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="2" t="s">
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="3" t="s">
         <v>6</v>
       </c>
       <c r="H11" s="4"/>
@@ -1264,14 +1405,14 @@
       <c r="R11" s="28"/>
     </row>
     <row r="12" spans="1:18" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="23"/>
-      <c r="B12" s="24"/>
-      <c r="C12" s="25"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
+      <c r="A12" s="14"/>
+      <c r="B12" s="15"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
       <c r="G12" s="5"/>
-      <c r="H12" s="7"/>
+      <c r="H12" s="6"/>
       <c r="I12" s="29"/>
       <c r="J12" s="30"/>
       <c r="K12" s="30"/>
@@ -1284,17 +1425,17 @@
       <c r="R12" s="31"/>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A13" s="8">
+      <c r="A13" s="10">
         <v>46104</v>
       </c>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1" t="s">
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="2" t="s">
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="3" t="s">
         <v>7</v>
       </c>
       <c r="H13" s="4"/>
@@ -1311,15 +1452,15 @@
       <c r="Q13" s="27"/>
       <c r="R13" s="28"/>
     </row>
-    <row r="14" spans="1:18" ht="104.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
+    <row r="14" spans="1:18" ht="105.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="9"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
       <c r="G14" s="5"/>
-      <c r="H14" s="7"/>
+      <c r="H14" s="6"/>
       <c r="I14" s="29"/>
       <c r="J14" s="30"/>
       <c r="K14" s="30"/>
@@ -1332,46 +1473,52 @@
       <c r="R14" s="31"/>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="2" t="s">
+      <c r="A15" s="10">
+        <v>46115</v>
+      </c>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="3" t="s">
         <v>8</v>
       </c>
       <c r="H15" s="4"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
-      <c r="L15" s="3"/>
-      <c r="M15" s="3"/>
-      <c r="N15" s="3"/>
-      <c r="O15" s="3"/>
-      <c r="P15" s="3"/>
-      <c r="Q15" s="3"/>
-      <c r="R15" s="4"/>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
+      <c r="I15" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="J15" s="27"/>
+      <c r="K15" s="27"/>
+      <c r="L15" s="27"/>
+      <c r="M15" s="27"/>
+      <c r="N15" s="27"/>
+      <c r="O15" s="27"/>
+      <c r="P15" s="27"/>
+      <c r="Q15" s="27"/>
+      <c r="R15" s="28"/>
+    </row>
+    <row r="16" spans="1:18" ht="105.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="9"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
       <c r="G16" s="5"/>
-      <c r="H16" s="7"/>
-      <c r="I16" s="5"/>
-      <c r="J16" s="6"/>
-      <c r="K16" s="6"/>
-      <c r="L16" s="6"/>
-      <c r="M16" s="6"/>
-      <c r="N16" s="6"/>
-      <c r="O16" s="6"/>
-      <c r="P16" s="6"/>
-      <c r="Q16" s="6"/>
-      <c r="R16" s="7"/>
+      <c r="H16" s="6"/>
+      <c r="I16" s="29"/>
+      <c r="J16" s="30"/>
+      <c r="K16" s="30"/>
+      <c r="L16" s="30"/>
+      <c r="M16" s="30"/>
+      <c r="N16" s="30"/>
+      <c r="O16" s="30"/>
+      <c r="P16" s="30"/>
+      <c r="Q16" s="30"/>
+      <c r="R16" s="31"/>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A17" s="32"/>
@@ -1383,17 +1530,17 @@
       <c r="G17" s="33" t="s">
         <v>9</v>
       </c>
-      <c r="H17" s="34"/>
+      <c r="H17" s="35"/>
       <c r="I17" s="33"/>
-      <c r="J17" s="35"/>
-      <c r="K17" s="35"/>
-      <c r="L17" s="35"/>
-      <c r="M17" s="35"/>
-      <c r="N17" s="35"/>
-      <c r="O17" s="35"/>
-      <c r="P17" s="35"/>
-      <c r="Q17" s="35"/>
-      <c r="R17" s="34"/>
+      <c r="J17" s="34"/>
+      <c r="K17" s="34"/>
+      <c r="L17" s="34"/>
+      <c r="M17" s="34"/>
+      <c r="N17" s="34"/>
+      <c r="O17" s="34"/>
+      <c r="P17" s="34"/>
+      <c r="Q17" s="34"/>
+      <c r="R17" s="35"/>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A18" s="32"/>
@@ -1403,17 +1550,17 @@
       <c r="E18" s="32"/>
       <c r="F18" s="32"/>
       <c r="G18" s="36"/>
-      <c r="H18" s="37"/>
+      <c r="H18" s="38"/>
       <c r="I18" s="36"/>
-      <c r="J18" s="38"/>
-      <c r="K18" s="38"/>
-      <c r="L18" s="38"/>
-      <c r="M18" s="38"/>
-      <c r="N18" s="38"/>
-      <c r="O18" s="38"/>
-      <c r="P18" s="38"/>
-      <c r="Q18" s="38"/>
-      <c r="R18" s="37"/>
+      <c r="J18" s="37"/>
+      <c r="K18" s="37"/>
+      <c r="L18" s="37"/>
+      <c r="M18" s="37"/>
+      <c r="N18" s="37"/>
+      <c r="O18" s="37"/>
+      <c r="P18" s="37"/>
+      <c r="Q18" s="37"/>
+      <c r="R18" s="38"/>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A19" s="32"/>
@@ -1500,127 +1647,143 @@
       <c r="R22" s="32"/>
     </row>
     <row r="23" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="39"/>
-      <c r="B23" s="39"/>
-      <c r="C23" s="39"/>
-      <c r="D23" s="39"/>
-      <c r="E23" s="40"/>
-      <c r="F23" s="39"/>
-      <c r="G23" s="39"/>
-      <c r="H23" s="39"/>
-      <c r="I23" s="39"/>
-      <c r="J23" s="39"/>
-      <c r="K23" s="39"/>
-      <c r="L23" s="39"/>
-      <c r="M23" s="39"/>
-      <c r="N23" s="39"/>
-      <c r="O23" s="39"/>
-      <c r="P23" s="39"/>
-      <c r="Q23" s="39"/>
-      <c r="R23" s="39"/>
+      <c r="A23" s="1"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+      <c r="I23" s="1"/>
+      <c r="J23" s="1"/>
+      <c r="K23" s="1"/>
+      <c r="L23" s="1"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+      <c r="O23" s="1"/>
+      <c r="P23" s="1"/>
+      <c r="Q23" s="1"/>
+      <c r="R23" s="1"/>
     </row>
     <row r="24" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="39"/>
-      <c r="B24" s="39"/>
-      <c r="C24" s="39"/>
-      <c r="D24" s="39"/>
-      <c r="E24" s="39"/>
-      <c r="F24" s="39"/>
-      <c r="G24" s="39"/>
-      <c r="H24" s="39"/>
-      <c r="I24" s="39"/>
-      <c r="J24" s="39"/>
-      <c r="K24" s="39"/>
-      <c r="L24" s="39"/>
-      <c r="M24" s="39"/>
-      <c r="N24" s="39"/>
-      <c r="O24" s="39"/>
-      <c r="P24" s="39"/>
-      <c r="Q24" s="39"/>
-      <c r="R24" s="39"/>
+      <c r="A24" s="1"/>
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="1"/>
+      <c r="H24" s="1"/>
+      <c r="I24" s="1"/>
+      <c r="J24" s="1"/>
+      <c r="K24" s="1"/>
+      <c r="L24" s="1"/>
+      <c r="M24" s="1"/>
+      <c r="N24" s="1"/>
+      <c r="O24" s="1"/>
+      <c r="P24" s="1"/>
+      <c r="Q24" s="1"/>
+      <c r="R24" s="1"/>
     </row>
     <row r="25" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="41"/>
-      <c r="B25" s="39"/>
-      <c r="C25" s="39"/>
-      <c r="D25" s="39"/>
-      <c r="E25" s="39"/>
-      <c r="F25" s="39"/>
-      <c r="G25" s="39"/>
-      <c r="H25" s="39"/>
-      <c r="I25" s="39"/>
-      <c r="J25" s="39"/>
-      <c r="K25" s="39"/>
-      <c r="L25" s="39"/>
-      <c r="M25" s="39"/>
-      <c r="N25" s="39"/>
-      <c r="O25" s="39"/>
-      <c r="P25" s="39"/>
-      <c r="Q25" s="39"/>
-      <c r="R25" s="39"/>
+      <c r="A25" s="2"/>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1"/>
+      <c r="H25" s="1"/>
+      <c r="I25" s="1"/>
+      <c r="J25" s="1"/>
+      <c r="K25" s="1"/>
+      <c r="L25" s="1"/>
+      <c r="M25" s="1"/>
+      <c r="N25" s="1"/>
+      <c r="O25" s="1"/>
+      <c r="P25" s="1"/>
+      <c r="Q25" s="1"/>
+      <c r="R25" s="1"/>
     </row>
     <row r="26" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="39"/>
-      <c r="B26" s="39"/>
-      <c r="C26" s="39"/>
-      <c r="D26" s="39"/>
-      <c r="E26" s="39"/>
-      <c r="F26" s="39"/>
-      <c r="G26" s="39"/>
-      <c r="H26" s="39"/>
-      <c r="I26" s="39"/>
-      <c r="J26" s="39"/>
-      <c r="K26" s="39"/>
-      <c r="L26" s="39"/>
-      <c r="M26" s="39"/>
-      <c r="N26" s="39"/>
-      <c r="O26" s="39"/>
-      <c r="P26" s="39"/>
-      <c r="Q26" s="39"/>
-      <c r="R26" s="39"/>
+      <c r="A26" s="1"/>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+      <c r="I26" s="1"/>
+      <c r="J26" s="1"/>
+      <c r="K26" s="1"/>
+      <c r="L26" s="1"/>
+      <c r="M26" s="1"/>
+      <c r="N26" s="1"/>
+      <c r="O26" s="1"/>
+      <c r="P26" s="1"/>
+      <c r="Q26" s="1"/>
+      <c r="R26" s="1"/>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A27" s="41"/>
-      <c r="B27" s="39"/>
-      <c r="C27" s="39"/>
-      <c r="D27" s="39"/>
-      <c r="E27" s="39"/>
-      <c r="F27" s="39"/>
-      <c r="G27" s="39"/>
-      <c r="H27" s="39"/>
-      <c r="I27" s="39"/>
-      <c r="J27" s="39"/>
-      <c r="K27" s="39"/>
-      <c r="L27" s="39"/>
-      <c r="M27" s="39"/>
-      <c r="N27" s="39"/>
-      <c r="O27" s="39"/>
-      <c r="P27" s="39"/>
-      <c r="Q27" s="39"/>
-      <c r="R27" s="39"/>
+      <c r="A27" s="2"/>
+      <c r="B27" s="1"/>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+      <c r="F27" s="1"/>
+      <c r="G27" s="1"/>
+      <c r="H27" s="1"/>
+      <c r="I27" s="1"/>
+      <c r="J27" s="1"/>
+      <c r="K27" s="1"/>
+      <c r="L27" s="1"/>
+      <c r="M27" s="1"/>
+      <c r="N27" s="1"/>
+      <c r="O27" s="1"/>
+      <c r="P27" s="1"/>
+      <c r="Q27" s="1"/>
+      <c r="R27" s="1"/>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A28" s="39"/>
-      <c r="B28" s="39"/>
-      <c r="C28" s="39"/>
-      <c r="D28" s="39"/>
-      <c r="E28" s="39"/>
-      <c r="F28" s="39"/>
-      <c r="G28" s="39"/>
-      <c r="H28" s="39"/>
-      <c r="I28" s="39"/>
-      <c r="J28" s="39"/>
-      <c r="K28" s="39"/>
-      <c r="L28" s="39"/>
-      <c r="M28" s="39"/>
-      <c r="N28" s="39"/>
-      <c r="O28" s="39"/>
-      <c r="P28" s="39"/>
-      <c r="Q28" s="39"/>
-      <c r="R28" s="39"/>
+      <c r="A28" s="1"/>
+      <c r="B28" s="1"/>
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
+      <c r="J28" s="1"/>
+      <c r="K28" s="1"/>
+      <c r="L28" s="1"/>
+      <c r="M28" s="1"/>
+      <c r="N28" s="1"/>
+      <c r="O28" s="1"/>
+      <c r="P28" s="1"/>
+      <c r="Q28" s="1"/>
+      <c r="R28" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="33">
+    <mergeCell ref="A17:C18"/>
+    <mergeCell ref="I17:R18"/>
+    <mergeCell ref="I19:R20"/>
+    <mergeCell ref="I21:R22"/>
+    <mergeCell ref="G17:H18"/>
+    <mergeCell ref="G19:H20"/>
+    <mergeCell ref="G21:H22"/>
+    <mergeCell ref="D21:F22"/>
+    <mergeCell ref="A19:C20"/>
+    <mergeCell ref="A21:C22"/>
+    <mergeCell ref="D17:F18"/>
+    <mergeCell ref="D19:F20"/>
+    <mergeCell ref="I11:R12"/>
+    <mergeCell ref="I13:R14"/>
+    <mergeCell ref="G3:H8"/>
+    <mergeCell ref="G9:H10"/>
+    <mergeCell ref="G11:H12"/>
     <mergeCell ref="G15:H16"/>
     <mergeCell ref="G13:H14"/>
     <mergeCell ref="I15:R16"/>
@@ -1637,23 +1800,6 @@
     <mergeCell ref="A15:C16"/>
     <mergeCell ref="I3:R8"/>
     <mergeCell ref="I9:R10"/>
-    <mergeCell ref="I11:R12"/>
-    <mergeCell ref="I13:R14"/>
-    <mergeCell ref="G3:H8"/>
-    <mergeCell ref="G9:H10"/>
-    <mergeCell ref="G11:H12"/>
-    <mergeCell ref="A17:C18"/>
-    <mergeCell ref="I17:R18"/>
-    <mergeCell ref="I19:R20"/>
-    <mergeCell ref="I21:R22"/>
-    <mergeCell ref="G17:H18"/>
-    <mergeCell ref="G19:H20"/>
-    <mergeCell ref="G21:H22"/>
-    <mergeCell ref="D21:F22"/>
-    <mergeCell ref="A19:C20"/>
-    <mergeCell ref="A21:C22"/>
-    <mergeCell ref="D17:F18"/>
-    <mergeCell ref="D19:F20"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>